<commit_message>
Auto commit - 10291713
</commit_message>
<xml_diff>
--- a/IM/202510_Service_Count_Report.xlsx
+++ b/IM/202510_Service_Count_Report.xlsx
@@ -275,10 +275,10 @@
     <t>台北市士林區德行西路100號</t>
   </si>
   <si>
+    <t>PM抄表</t>
+  </si>
+  <si>
     <t>服務</t>
-  </si>
-  <si>
-    <t>PM抄表</t>
   </si>
   <si>
     <t>10:27:00</t>
@@ -2763,22 +2763,22 @@
 換下 8187000916</t>
   </si>
   <si>
+    <t>THILF0D349</t>
+  </si>
+  <si>
+    <t>新北市板橋區重慶路245巷61號</t>
+  </si>
+  <si>
+    <t>板橋成都店</t>
+  </si>
+  <si>
     <t>15:45:00</t>
   </si>
   <si>
-    <t>THILF0D349</t>
-  </si>
-  <si>
-    <t>新北市板橋區重慶路245巷61號</t>
-  </si>
-  <si>
-    <t>板橋成都店</t>
+    <t>驅動修復測試正常，請門市觀察中</t>
   </si>
   <si>
     <t>PMQ4 L99</t>
-  </si>
-  <si>
-    <t>驅動修復測試正常，請門市觀察中</t>
   </si>
   <si>
     <t>TX30000054</t>
@@ -3872,7 +3872,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>2025102727</v>
+        <v>2025102728</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
@@ -3909,7 +3909,7 @@
       </c>
       <c r="N10" s="6"/>
       <c r="O10" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P10" s="3"/>
       <c r="Q10" s="3">
@@ -3918,9 +3918,7 @@
       <c r="R10" s="3">
         <v>2018</v>
       </c>
-      <c r="S10" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S10" s="3"/>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
@@ -3928,7 +3926,7 @@
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
       <c r="Z10" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA10" s="3" t="s">
         <v>40</v>
@@ -3942,7 +3940,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="7">
-        <v>2025102728</v>
+        <v>2025102727</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
@@ -3979,7 +3977,7 @@
       </c>
       <c r="N11" s="8"/>
       <c r="O11" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P11" s="7"/>
       <c r="Q11" s="7">
@@ -3988,7 +3986,9 @@
       <c r="R11" s="7">
         <v>2018</v>
       </c>
-      <c r="S11" s="7"/>
+      <c r="S11" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T11" s="7"/>
       <c r="U11" s="7"/>
       <c r="V11" s="7"/>
@@ -3996,7 +3996,7 @@
       <c r="X11" s="7"/>
       <c r="Y11" s="7"/>
       <c r="Z11" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA11" s="7" t="s">
         <v>40</v>
@@ -4117,7 +4117,7 @@
         <v>94</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P13" s="7"/>
       <c r="Q13" s="7">
@@ -4136,7 +4136,7 @@
       <c r="X13" s="7"/>
       <c r="Y13" s="7"/>
       <c r="Z13" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA13" s="7" t="s">
         <v>40</v>
@@ -4206,7 +4206,7 @@
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA14" s="3" t="s">
         <v>40</v>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="N16" s="6"/>
       <c r="O16" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P16" s="3"/>
       <c r="Q16" s="3">
@@ -4344,7 +4344,7 @@
       <c r="X16" s="3"/>
       <c r="Y16" s="3"/>
       <c r="Z16" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA16" s="3" t="s">
         <v>40</v>
@@ -4412,7 +4412,7 @@
       <c r="X17" s="7"/>
       <c r="Y17" s="7"/>
       <c r="Z17" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA17" s="7" t="s">
         <v>40</v>
@@ -4424,7 +4424,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>2025101693</v>
+        <v>2025101694</v>
       </c>
       <c r="C18" s="3">
         <v>1</v>
@@ -4463,7 +4463,7 @@
         <v>108</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P18" s="3"/>
       <c r="Q18" s="3">
@@ -4472,9 +4472,7 @@
       <c r="R18" s="3">
         <v>2479</v>
       </c>
-      <c r="S18" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S18" s="3"/>
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
@@ -4482,7 +4480,7 @@
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
       <c r="Z18" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA18" s="3" t="s">
         <v>40</v>
@@ -4496,7 +4494,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="7">
-        <v>2025101694</v>
+        <v>2025101693</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -4535,7 +4533,7 @@
         <v>108</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P19" s="7"/>
       <c r="Q19" s="7">
@@ -4544,7 +4542,9 @@
       <c r="R19" s="7">
         <v>2479</v>
       </c>
-      <c r="S19" s="7"/>
+      <c r="S19" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T19" s="7"/>
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
@@ -4552,7 +4552,7 @@
       <c r="X19" s="7"/>
       <c r="Y19" s="7"/>
       <c r="Z19" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA19" s="7" t="s">
         <v>40</v>
@@ -4603,7 +4603,7 @@
         <v>108</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P20" s="3"/>
       <c r="Q20" s="3">
@@ -4622,7 +4622,7 @@
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
       <c r="Z20" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA20" s="3" t="s">
         <v>40</v>
@@ -4692,7 +4692,7 @@
       <c r="X21" s="7"/>
       <c r="Y21" s="7"/>
       <c r="Z21" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA21" s="7" t="s">
         <v>40</v>
@@ -4743,7 +4743,7 @@
         <v>52</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P22" s="3"/>
       <c r="Q22" s="3">
@@ -4762,7 +4762,7 @@
       <c r="X22" s="3"/>
       <c r="Y22" s="3"/>
       <c r="Z22" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA22" s="3" t="s">
         <v>40</v>
@@ -4832,7 +4832,7 @@
       <c r="X23" s="7"/>
       <c r="Y23" s="7"/>
       <c r="Z23" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA23" s="7" t="s">
         <v>40</v>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="N24" s="6"/>
       <c r="O24" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P24" s="3"/>
       <c r="Q24" s="3"/>
@@ -4972,7 +4972,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>2025101688</v>
+        <v>2025101689</v>
       </c>
       <c r="C26" s="3">
         <v>1</v>
@@ -5011,16 +5011,14 @@
         <v>128</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
       <c r="R26" s="3">
         <v>1845</v>
       </c>
-      <c r="S26" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
@@ -5028,7 +5026,7 @@
       <c r="X26" s="3"/>
       <c r="Y26" s="3"/>
       <c r="Z26" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA26" s="3" t="s">
         <v>40</v>
@@ -5042,7 +5040,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="7">
-        <v>2025101689</v>
+        <v>2025101688</v>
       </c>
       <c r="C27" s="7">
         <v>1</v>
@@ -5081,14 +5079,16 @@
         <v>128</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P27" s="7"/>
       <c r="Q27" s="7"/>
       <c r="R27" s="7">
         <v>1845</v>
       </c>
-      <c r="S27" s="7"/>
+      <c r="S27" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T27" s="7"/>
       <c r="U27" s="7"/>
       <c r="V27" s="7"/>
@@ -5096,7 +5096,7 @@
       <c r="X27" s="7"/>
       <c r="Y27" s="7"/>
       <c r="Z27" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA27" s="7" t="s">
         <v>40</v>
@@ -5213,7 +5213,7 @@
         <v>30</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P29" s="7"/>
       <c r="Q29" s="7"/>
@@ -5230,7 +5230,7 @@
       <c r="X29" s="7"/>
       <c r="Y29" s="7"/>
       <c r="Z29" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA29" s="7"/>
       <c r="AB29" s="7"/>
@@ -5294,7 +5294,7 @@
       <c r="X30" s="3"/>
       <c r="Y30" s="3"/>
       <c r="Z30" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA30" s="3" t="s">
         <v>40</v>
@@ -5345,7 +5345,7 @@
         <v>30</v>
       </c>
       <c r="O31" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P31" s="7"/>
       <c r="Q31" s="7"/>
@@ -5413,7 +5413,7 @@
         <v>30</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
@@ -5430,7 +5430,7 @@
       <c r="X32" s="3"/>
       <c r="Y32" s="3"/>
       <c r="Z32" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA32" s="3" t="s">
         <v>40</v>
@@ -5498,7 +5498,7 @@
       <c r="X33" s="7"/>
       <c r="Y33" s="7"/>
       <c r="Z33" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA33" s="7" t="s">
         <v>40</v>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="N34" s="6"/>
       <c r="O34" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="N36" s="6"/>
       <c r="O36" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
@@ -5745,7 +5745,7 @@
         <v>159</v>
       </c>
       <c r="O37" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P37" s="7"/>
       <c r="Q37" s="7"/>
@@ -5762,7 +5762,7 @@
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
       <c r="Z37" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA37" s="7" t="s">
         <v>40</v>
@@ -5830,7 +5830,7 @@
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
       <c r="Z38" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA38" s="3" t="s">
         <v>40</v>
@@ -5842,7 +5842,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="7">
-        <v>2025102577</v>
+        <v>2025102578</v>
       </c>
       <c r="C39" s="7">
         <v>1</v>
@@ -5881,16 +5881,14 @@
         <v>30</v>
       </c>
       <c r="O39" s="7" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P39" s="7"/>
       <c r="Q39" s="7"/>
       <c r="R39" s="7">
         <v>36832</v>
       </c>
-      <c r="S39" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S39" s="7"/>
       <c r="T39" s="7"/>
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
@@ -5898,17 +5896,21 @@
       <c r="X39" s="7"/>
       <c r="Y39" s="7"/>
       <c r="Z39" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA39" s="7"/>
-      <c r="AB39" s="7"/>
+        <v>81</v>
+      </c>
+      <c r="AA39" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB39" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="40" spans="1:28">
       <c r="A40" s="3">
         <v>38</v>
       </c>
       <c r="B40" s="3">
-        <v>2025102578</v>
+        <v>2025102577</v>
       </c>
       <c r="C40" s="3">
         <v>1</v>
@@ -5947,14 +5949,16 @@
         <v>30</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
       <c r="R40" s="3">
         <v>36832</v>
       </c>
-      <c r="S40" s="3"/>
+      <c r="S40" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
       <c r="V40" s="3"/>
@@ -5962,11 +5966,9 @@
       <c r="X40" s="3"/>
       <c r="Y40" s="3"/>
       <c r="Z40" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA40" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="AA40" s="3"/>
       <c r="AB40" s="3"/>
     </row>
     <row r="41" spans="1:28">
@@ -6013,7 +6015,7 @@
         <v>169</v>
       </c>
       <c r="O41" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P41" s="7"/>
       <c r="Q41" s="7"/>
@@ -6030,7 +6032,7 @@
       <c r="X41" s="7"/>
       <c r="Y41" s="7"/>
       <c r="Z41" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA41" s="7" t="s">
         <v>40</v>
@@ -6098,7 +6100,7 @@
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
       <c r="Z42" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA42" s="3" t="s">
         <v>40</v>
@@ -6147,7 +6149,7 @@
       </c>
       <c r="N43" s="8"/>
       <c r="O43" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P43" s="7"/>
       <c r="Q43" s="7"/>
@@ -6164,7 +6166,7 @@
       <c r="X43" s="7"/>
       <c r="Y43" s="7"/>
       <c r="Z43" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA43" s="7" t="s">
         <v>40</v>
@@ -6230,7 +6232,7 @@
       <c r="X44" s="3"/>
       <c r="Y44" s="3"/>
       <c r="Z44" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA44" s="3" t="s">
         <v>40</v>
@@ -6279,7 +6281,7 @@
       </c>
       <c r="N45" s="8"/>
       <c r="O45" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
@@ -6349,7 +6351,7 @@
         <v>180</v>
       </c>
       <c r="O46" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P46" s="3"/>
       <c r="Q46" s="3"/>
@@ -6366,7 +6368,7 @@
       <c r="X46" s="3"/>
       <c r="Y46" s="3"/>
       <c r="Z46" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA46" s="3" t="s">
         <v>40</v>
@@ -6434,7 +6436,7 @@
       <c r="X47" s="7"/>
       <c r="Y47" s="7"/>
       <c r="Z47" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA47" s="7" t="s">
         <v>40</v>
@@ -6485,7 +6487,7 @@
         <v>30</v>
       </c>
       <c r="O48" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P48" s="3"/>
       <c r="Q48" s="3"/>
@@ -6502,7 +6504,7 @@
       <c r="X48" s="3"/>
       <c r="Y48" s="3"/>
       <c r="Z48" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA48" s="3"/>
       <c r="AB48" s="3"/>
@@ -6566,7 +6568,7 @@
       <c r="X49" s="7"/>
       <c r="Y49" s="7"/>
       <c r="Z49" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA49" s="7" t="s">
         <v>40</v>
@@ -6617,7 +6619,7 @@
         <v>191</v>
       </c>
       <c r="O50" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P50" s="3"/>
       <c r="Q50" s="3">
@@ -6689,7 +6691,7 @@
         <v>159</v>
       </c>
       <c r="O51" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P51" s="7"/>
       <c r="Q51" s="7">
@@ -6708,7 +6710,7 @@
       <c r="X51" s="7"/>
       <c r="Y51" s="7"/>
       <c r="Z51" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA51" s="7" t="s">
         <v>40</v>
@@ -6778,7 +6780,7 @@
       <c r="X52" s="3"/>
       <c r="Y52" s="3"/>
       <c r="Z52" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA52" s="3" t="s">
         <v>40</v>
@@ -6829,7 +6831,7 @@
         <v>159</v>
       </c>
       <c r="O53" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P53" s="7"/>
       <c r="Q53" s="7">
@@ -6901,7 +6903,7 @@
         <v>206</v>
       </c>
       <c r="O54" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P54" s="3"/>
       <c r="Q54" s="3">
@@ -6920,7 +6922,7 @@
       <c r="X54" s="3"/>
       <c r="Y54" s="3"/>
       <c r="Z54" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA54" s="3" t="s">
         <v>40</v>
@@ -6990,7 +6992,7 @@
       <c r="X55" s="7"/>
       <c r="Y55" s="7"/>
       <c r="Z55" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA55" s="7" t="s">
         <v>40</v>
@@ -7179,7 +7181,7 @@
         <v>223</v>
       </c>
       <c r="O58" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P58" s="3"/>
       <c r="Q58" s="3">
@@ -7198,7 +7200,7 @@
       <c r="X58" s="3"/>
       <c r="Y58" s="3"/>
       <c r="Z58" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA58" s="3" t="s">
         <v>40</v>
@@ -7268,7 +7270,7 @@
       <c r="X59" s="7"/>
       <c r="Y59" s="7"/>
       <c r="Z59" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA59" s="7" t="s">
         <v>40</v>
@@ -7385,7 +7387,7 @@
       </c>
       <c r="N61" s="8"/>
       <c r="O61" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P61" s="7"/>
       <c r="Q61" s="7"/>
@@ -7480,7 +7482,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="7">
-        <v>2025103003</v>
+        <v>2025103002</v>
       </c>
       <c r="C63" s="7">
         <v>1</v>
@@ -7519,14 +7521,16 @@
         <v>236</v>
       </c>
       <c r="O63" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P63" s="7"/>
       <c r="Q63" s="7"/>
       <c r="R63" s="7">
         <v>142499</v>
       </c>
-      <c r="S63" s="7"/>
+      <c r="S63" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T63" s="7"/>
       <c r="U63" s="7"/>
       <c r="V63" s="7"/>
@@ -7534,7 +7538,7 @@
       <c r="X63" s="7"/>
       <c r="Y63" s="7"/>
       <c r="Z63" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA63" s="7" t="s">
         <v>40</v>
@@ -7548,7 +7552,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="3">
-        <v>2025103002</v>
+        <v>2025103003</v>
       </c>
       <c r="C64" s="3">
         <v>1</v>
@@ -7587,16 +7591,14 @@
         <v>236</v>
       </c>
       <c r="O64" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P64" s="3"/>
       <c r="Q64" s="3"/>
       <c r="R64" s="3">
         <v>142499</v>
       </c>
-      <c r="S64" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S64" s="3"/>
       <c r="T64" s="3"/>
       <c r="U64" s="3"/>
       <c r="V64" s="3"/>
@@ -7604,7 +7606,7 @@
       <c r="X64" s="3"/>
       <c r="Y64" s="3"/>
       <c r="Z64" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA64" s="3" t="s">
         <v>40</v>
@@ -7655,7 +7657,7 @@
         <v>240</v>
       </c>
       <c r="O65" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P65" s="7"/>
       <c r="Q65" s="7"/>
@@ -7672,7 +7674,7 @@
       <c r="X65" s="7"/>
       <c r="Y65" s="7"/>
       <c r="Z65" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA65" s="7" t="s">
         <v>40</v>
@@ -7740,7 +7742,7 @@
       <c r="X66" s="3"/>
       <c r="Y66" s="3"/>
       <c r="Z66" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA66" s="3" t="s">
         <v>40</v>
@@ -7787,7 +7789,7 @@
         <v>247</v>
       </c>
       <c r="O67" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P67" s="7"/>
       <c r="Q67" s="7"/>
@@ -7853,7 +7855,7 @@
         <v>254</v>
       </c>
       <c r="O68" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P68" s="3"/>
       <c r="Q68" s="3"/>
@@ -7919,7 +7921,7 @@
         <v>259</v>
       </c>
       <c r="O69" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P69" s="7"/>
       <c r="Q69" s="7"/>
@@ -8051,7 +8053,7 @@
         <v>268</v>
       </c>
       <c r="O71" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P71" s="7"/>
       <c r="Q71" s="7"/>
@@ -8117,7 +8119,7 @@
         <v>273</v>
       </c>
       <c r="O72" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P72" s="3"/>
       <c r="Q72" s="3"/>
@@ -8183,7 +8185,7 @@
         <v>277</v>
       </c>
       <c r="O73" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P73" s="7"/>
       <c r="Q73" s="7"/>
@@ -8317,7 +8319,7 @@
         <v>286</v>
       </c>
       <c r="O75" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P75" s="7"/>
       <c r="Q75" s="7"/>
@@ -8383,7 +8385,7 @@
         <v>289</v>
       </c>
       <c r="O76" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P76" s="3"/>
       <c r="Q76" s="3"/>
@@ -8449,7 +8451,7 @@
         <v>294</v>
       </c>
       <c r="O77" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P77" s="7"/>
       <c r="Q77" s="7"/>
@@ -8515,7 +8517,7 @@
         <v>297</v>
       </c>
       <c r="O78" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P78" s="3"/>
       <c r="Q78" s="3"/>
@@ -8581,7 +8583,7 @@
         <v>297</v>
       </c>
       <c r="O79" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P79" s="7"/>
       <c r="Q79" s="7"/>
@@ -8715,7 +8717,7 @@
         <v>303</v>
       </c>
       <c r="O81" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P81" s="7"/>
       <c r="Q81" s="7"/>
@@ -8779,7 +8781,7 @@
         <v>311</v>
       </c>
       <c r="O82" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P82" s="3"/>
       <c r="Q82" s="3"/>
@@ -8845,7 +8847,7 @@
         <v>316</v>
       </c>
       <c r="O83" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P83" s="7"/>
       <c r="Q83" s="7"/>
@@ -8911,7 +8913,7 @@
         <v>321</v>
       </c>
       <c r="O84" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P84" s="3"/>
       <c r="Q84" s="3"/>
@@ -8977,7 +8979,7 @@
         <v>325</v>
       </c>
       <c r="O85" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P85" s="7"/>
       <c r="Q85" s="7"/>
@@ -9179,7 +9181,7 @@
         <v>343</v>
       </c>
       <c r="O88" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P88" s="3"/>
       <c r="Q88" s="3"/>
@@ -9381,7 +9383,7 @@
         <v>352</v>
       </c>
       <c r="O91" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P91" s="7"/>
       <c r="Q91" s="7"/>
@@ -9785,7 +9787,7 @@
         <v>366</v>
       </c>
       <c r="O97" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P97" s="7"/>
       <c r="Q97" s="7"/>
@@ -9849,7 +9851,7 @@
         <v>374</v>
       </c>
       <c r="O98" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P98" s="3"/>
       <c r="Q98" s="3"/>
@@ -9915,7 +9917,7 @@
         <v>377</v>
       </c>
       <c r="O99" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P99" s="7"/>
       <c r="Q99" s="7"/>
@@ -9981,7 +9983,7 @@
         <v>381</v>
       </c>
       <c r="O100" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P100" s="3"/>
       <c r="Q100" s="3"/>
@@ -10115,7 +10117,7 @@
         <v>388</v>
       </c>
       <c r="O102" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P102" s="3"/>
       <c r="Q102" s="3"/>
@@ -10181,7 +10183,7 @@
         <v>391</v>
       </c>
       <c r="O103" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P103" s="7"/>
       <c r="Q103" s="7"/>
@@ -10247,7 +10249,7 @@
         <v>395</v>
       </c>
       <c r="O104" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P104" s="3"/>
       <c r="Q104" s="3"/>
@@ -10313,7 +10315,7 @@
         <v>400</v>
       </c>
       <c r="O105" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P105" s="7"/>
       <c r="Q105" s="7"/>
@@ -10379,7 +10381,7 @@
         <v>404</v>
       </c>
       <c r="O106" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P106" s="3"/>
       <c r="Q106" s="3"/>
@@ -10445,7 +10447,7 @@
         <v>408</v>
       </c>
       <c r="O107" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P107" s="7"/>
       <c r="Q107" s="7"/>
@@ -10511,7 +10513,7 @@
         <v>412</v>
       </c>
       <c r="O108" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P108" s="3"/>
       <c r="Q108" s="3"/>
@@ -10577,7 +10579,7 @@
         <v>417</v>
       </c>
       <c r="O109" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P109" s="7"/>
       <c r="Q109" s="7"/>
@@ -10643,7 +10645,7 @@
         <v>421</v>
       </c>
       <c r="O110" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P110" s="3"/>
       <c r="Q110" s="3"/>
@@ -10709,7 +10711,7 @@
         <v>424</v>
       </c>
       <c r="O111" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P111" s="7"/>
       <c r="Q111" s="7"/>
@@ -10843,7 +10845,7 @@
         <v>427</v>
       </c>
       <c r="O113" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P113" s="7"/>
       <c r="Q113" s="7"/>
@@ -10909,7 +10911,7 @@
         <v>433</v>
       </c>
       <c r="O114" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P114" s="3"/>
       <c r="Q114" s="3"/>
@@ -10975,7 +10977,7 @@
         <v>437</v>
       </c>
       <c r="O115" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P115" s="7"/>
       <c r="Q115" s="7"/>
@@ -11041,7 +11043,7 @@
         <v>437</v>
       </c>
       <c r="O116" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P116" s="3"/>
       <c r="Q116" s="3"/>
@@ -11107,7 +11109,7 @@
         <v>441</v>
       </c>
       <c r="O117" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P117" s="7"/>
       <c r="Q117" s="7"/>
@@ -11173,7 +11175,7 @@
         <v>446</v>
       </c>
       <c r="O118" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P118" s="3"/>
       <c r="Q118" s="3"/>
@@ -11307,7 +11309,7 @@
         <v>446</v>
       </c>
       <c r="O120" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P120" s="3"/>
       <c r="Q120" s="3"/>
@@ -11373,7 +11375,7 @@
         <v>454</v>
       </c>
       <c r="O121" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P121" s="7"/>
       <c r="Q121" s="7"/>
@@ -11439,7 +11441,7 @@
         <v>458</v>
       </c>
       <c r="O122" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P122" s="3"/>
       <c r="Q122" s="3"/>
@@ -11505,7 +11507,7 @@
         <v>463</v>
       </c>
       <c r="O123" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P123" s="7"/>
       <c r="Q123" s="7"/>
@@ -11639,7 +11641,7 @@
         <v>466</v>
       </c>
       <c r="O125" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P125" s="7"/>
       <c r="Q125" s="7"/>
@@ -11705,7 +11707,7 @@
         <v>471</v>
       </c>
       <c r="O126" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P126" s="3"/>
       <c r="Q126" s="3"/>
@@ -11771,7 +11773,7 @@
         <v>474</v>
       </c>
       <c r="O127" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P127" s="7"/>
       <c r="Q127" s="7"/>
@@ -11905,7 +11907,7 @@
         <v>480</v>
       </c>
       <c r="O129" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P129" s="7"/>
       <c r="Q129" s="7"/>
@@ -11969,7 +11971,7 @@
         <v>485</v>
       </c>
       <c r="O130" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P130" s="3"/>
       <c r="Q130" s="3"/>
@@ -12039,7 +12041,7 @@
         <v>491</v>
       </c>
       <c r="O131" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P131" s="7"/>
       <c r="Q131" s="7">
@@ -12179,7 +12181,7 @@
         <v>491</v>
       </c>
       <c r="O133" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P133" s="7"/>
       <c r="Q133" s="7">
@@ -12251,7 +12253,7 @@
         <v>499</v>
       </c>
       <c r="O134" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P134" s="3"/>
       <c r="Q134" s="3">
@@ -12385,7 +12387,7 @@
       </c>
       <c r="N136" s="6"/>
       <c r="O136" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P136" s="3"/>
       <c r="Q136" s="3">
@@ -12523,7 +12525,7 @@
         <v>507</v>
       </c>
       <c r="O138" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P138" s="3"/>
       <c r="Q138" s="3">
@@ -12595,7 +12597,7 @@
         <v>507</v>
       </c>
       <c r="O139" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P139" s="7"/>
       <c r="Q139" s="7">
@@ -12805,7 +12807,7 @@
         <v>514</v>
       </c>
       <c r="O142" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P142" s="3"/>
       <c r="Q142" s="3">
@@ -12941,7 +12943,7 @@
         <v>518</v>
       </c>
       <c r="O144" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P144" s="3"/>
       <c r="Q144" s="3">
@@ -13077,7 +13079,7 @@
         <v>521</v>
       </c>
       <c r="O146" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P146" s="3"/>
       <c r="Q146" s="3">
@@ -13149,7 +13151,7 @@
         <v>521</v>
       </c>
       <c r="O147" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P147" s="7"/>
       <c r="Q147" s="7">
@@ -13285,7 +13287,7 @@
         <v>525</v>
       </c>
       <c r="O149" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P149" s="7">
         <v>6677</v>
@@ -13429,7 +13431,7 @@
         <v>528</v>
       </c>
       <c r="O151" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P151" s="7">
         <v>1800</v>
@@ -13573,7 +13575,7 @@
         <v>532</v>
       </c>
       <c r="O153" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P153" s="7"/>
       <c r="Q153" s="7">
@@ -13713,7 +13715,7 @@
         <v>535</v>
       </c>
       <c r="O155" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P155" s="7">
         <v>117</v>
@@ -13857,7 +13859,7 @@
         <v>539</v>
       </c>
       <c r="O157" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P157" s="7"/>
       <c r="Q157" s="7">
@@ -14094,7 +14096,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="7">
-        <v>2025100085</v>
+        <v>2025100084</v>
       </c>
       <c r="C161" s="7">
         <v>1</v>
@@ -14133,7 +14135,7 @@
         <v>532</v>
       </c>
       <c r="O161" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P161" s="7"/>
       <c r="Q161" s="7">
@@ -14142,7 +14144,9 @@
       <c r="R161" s="7">
         <v>400</v>
       </c>
-      <c r="S161" s="7"/>
+      <c r="S161" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T161" s="7"/>
       <c r="U161" s="7"/>
       <c r="V161" s="7"/>
@@ -14164,7 +14168,7 @@
         <v>160</v>
       </c>
       <c r="B162" s="3">
-        <v>2025100084</v>
+        <v>2025100085</v>
       </c>
       <c r="C162" s="3">
         <v>1</v>
@@ -14203,7 +14207,7 @@
         <v>532</v>
       </c>
       <c r="O162" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P162" s="3"/>
       <c r="Q162" s="3">
@@ -14212,9 +14216,7 @@
       <c r="R162" s="3">
         <v>400</v>
       </c>
-      <c r="S162" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S162" s="3"/>
       <c r="T162" s="3"/>
       <c r="U162" s="3"/>
       <c r="V162" s="3"/>
@@ -14343,7 +14345,7 @@
         <v>547</v>
       </c>
       <c r="O164" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P164" s="3"/>
       <c r="Q164" s="3">
@@ -14479,7 +14481,7 @@
         <v>547</v>
       </c>
       <c r="O166" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P166" s="3"/>
       <c r="Q166" s="3">
@@ -14551,7 +14553,7 @@
         <v>550</v>
       </c>
       <c r="O167" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P167" s="7"/>
       <c r="Q167" s="7">
@@ -14648,7 +14650,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="7">
-        <v>2025101233</v>
+        <v>2025101232</v>
       </c>
       <c r="C169" s="7">
         <v>1</v>
@@ -14687,7 +14689,7 @@
         <v>554</v>
       </c>
       <c r="O169" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P169" s="7"/>
       <c r="Q169" s="7">
@@ -14696,7 +14698,9 @@
       <c r="R169" s="7">
         <v>1179</v>
       </c>
-      <c r="S169" s="7"/>
+      <c r="S169" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T169" s="7"/>
       <c r="U169" s="7"/>
       <c r="V169" s="7"/>
@@ -14706,19 +14710,15 @@
       <c r="Z169" s="8" t="s">
         <v>492</v>
       </c>
-      <c r="AA169" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="AB169" s="7">
-        <v>1</v>
-      </c>
+      <c r="AA169" s="7"/>
+      <c r="AB169" s="7"/>
     </row>
     <row r="170" spans="1:28">
       <c r="A170" s="3">
         <v>168</v>
       </c>
       <c r="B170" s="3">
-        <v>2025101232</v>
+        <v>2025101233</v>
       </c>
       <c r="C170" s="3">
         <v>1</v>
@@ -14757,7 +14757,7 @@
         <v>554</v>
       </c>
       <c r="O170" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P170" s="3"/>
       <c r="Q170" s="3">
@@ -14766,9 +14766,7 @@
       <c r="R170" s="3">
         <v>1179</v>
       </c>
-      <c r="S170" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S170" s="3"/>
       <c r="T170" s="3"/>
       <c r="U170" s="3"/>
       <c r="V170" s="3"/>
@@ -14778,7 +14776,9 @@
       <c r="Z170" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="AA170" s="3"/>
+      <c r="AA170" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="AB170" s="3"/>
     </row>
     <row r="171" spans="1:28">
@@ -15165,7 +15165,7 @@
         <v>569</v>
       </c>
       <c r="O176" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P176" s="3"/>
       <c r="Q176" s="3"/>
@@ -15303,7 +15303,7 @@
         <v>578</v>
       </c>
       <c r="O178" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P178" s="3"/>
       <c r="Q178" s="3"/>
@@ -15437,7 +15437,7 @@
       </c>
       <c r="N180" s="6"/>
       <c r="O180" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P180" s="3"/>
       <c r="Q180" s="3"/>
@@ -15571,7 +15571,7 @@
         <v>585</v>
       </c>
       <c r="O182" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P182" s="3"/>
       <c r="Q182" s="3"/>
@@ -15707,7 +15707,7 @@
         <v>585</v>
       </c>
       <c r="O184" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P184" s="3"/>
       <c r="Q184" s="3"/>
@@ -15843,7 +15843,7 @@
         <v>590</v>
       </c>
       <c r="O186" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P186" s="3"/>
       <c r="Q186" s="3"/>
@@ -15975,7 +15975,7 @@
         <v>590</v>
       </c>
       <c r="O188" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P188" s="3"/>
       <c r="Q188" s="3"/>
@@ -16111,7 +16111,7 @@
         <v>595</v>
       </c>
       <c r="O190" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P190" s="3"/>
       <c r="Q190" s="3"/>
@@ -16208,7 +16208,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="3">
-        <v>2025100369</v>
+        <v>2025100368</v>
       </c>
       <c r="C192" s="3">
         <v>1</v>
@@ -16247,14 +16247,16 @@
         <v>599</v>
       </c>
       <c r="O192" s="3" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P192" s="3"/>
       <c r="Q192" s="3"/>
       <c r="R192" s="3">
         <v>155192</v>
       </c>
-      <c r="S192" s="3"/>
+      <c r="S192" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T192" s="3"/>
       <c r="U192" s="3"/>
       <c r="V192" s="3"/>
@@ -16276,7 +16278,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="7">
-        <v>2025100368</v>
+        <v>2025100369</v>
       </c>
       <c r="C193" s="7">
         <v>1</v>
@@ -16315,16 +16317,14 @@
         <v>599</v>
       </c>
       <c r="O193" s="7" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P193" s="7"/>
       <c r="Q193" s="7"/>
       <c r="R193" s="7">
         <v>155192</v>
       </c>
-      <c r="S193" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S193" s="7"/>
       <c r="T193" s="7"/>
       <c r="U193" s="7"/>
       <c r="V193" s="7"/>
@@ -16383,7 +16383,7 @@
         <v>602</v>
       </c>
       <c r="O194" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P194" s="3"/>
       <c r="Q194" s="3"/>
@@ -16585,7 +16585,7 @@
       </c>
       <c r="N197" s="8"/>
       <c r="O197" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P197" s="7"/>
       <c r="Q197" s="7"/>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="N199" s="8"/>
       <c r="O199" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P199" s="7"/>
       <c r="Q199" s="7"/>
@@ -16787,7 +16787,7 @@
         <v>565</v>
       </c>
       <c r="O200" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P200" s="3"/>
       <c r="Q200" s="3"/>
@@ -16857,7 +16857,7 @@
         <v>565</v>
       </c>
       <c r="O201" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P201" s="7"/>
       <c r="Q201" s="7"/>
@@ -16927,7 +16927,7 @@
         <v>613</v>
       </c>
       <c r="O202" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P202" s="3"/>
       <c r="Q202" s="3"/>
@@ -17059,7 +17059,7 @@
         <v>617</v>
       </c>
       <c r="O204" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P204" s="3"/>
       <c r="Q204" s="3"/>
@@ -17191,7 +17191,7 @@
         <v>620</v>
       </c>
       <c r="O206" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P206" s="3"/>
       <c r="Q206" s="3"/>
@@ -17323,7 +17323,7 @@
         <v>532</v>
       </c>
       <c r="O208" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P208" s="3"/>
       <c r="Q208" s="3"/>
@@ -17459,7 +17459,7 @@
         <v>625</v>
       </c>
       <c r="O210" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P210" s="3"/>
       <c r="Q210" s="3"/>
@@ -17595,7 +17595,7 @@
         <v>628</v>
       </c>
       <c r="O212" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P212" s="3"/>
       <c r="Q212" s="3"/>
@@ -17731,7 +17731,7 @@
         <v>631</v>
       </c>
       <c r="O214" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P214" s="3"/>
       <c r="Q214" s="3"/>
@@ -17828,7 +17828,7 @@
         <v>214</v>
       </c>
       <c r="B216" s="3">
-        <v>2025100063</v>
+        <v>2025100064</v>
       </c>
       <c r="C216" s="3">
         <v>1</v>
@@ -17867,16 +17867,14 @@
         <v>634</v>
       </c>
       <c r="O216" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P216" s="3"/>
       <c r="Q216" s="3"/>
       <c r="R216" s="3">
         <v>2841</v>
       </c>
-      <c r="S216" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S216" s="3"/>
       <c r="T216" s="3"/>
       <c r="U216" s="3"/>
       <c r="V216" s="3"/>
@@ -17898,7 +17896,7 @@
         <v>215</v>
       </c>
       <c r="B217" s="7">
-        <v>2025100064</v>
+        <v>2025100063</v>
       </c>
       <c r="C217" s="7">
         <v>1</v>
@@ -17937,14 +17935,16 @@
         <v>634</v>
       </c>
       <c r="O217" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P217" s="7"/>
       <c r="Q217" s="7"/>
       <c r="R217" s="7">
         <v>2841</v>
       </c>
-      <c r="S217" s="7"/>
+      <c r="S217" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T217" s="7"/>
       <c r="U217" s="7"/>
       <c r="V217" s="7"/>
@@ -18003,7 +18003,7 @@
         <v>547</v>
       </c>
       <c r="O218" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P218" s="3"/>
       <c r="Q218" s="3"/>
@@ -18100,7 +18100,7 @@
         <v>218</v>
       </c>
       <c r="B220" s="3">
-        <v>2025102607</v>
+        <v>2025102606</v>
       </c>
       <c r="C220" s="3">
         <v>1</v>
@@ -18139,14 +18139,16 @@
         <v>634</v>
       </c>
       <c r="O220" s="3" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P220" s="3"/>
       <c r="Q220" s="3"/>
       <c r="R220" s="3">
         <v>1291</v>
       </c>
-      <c r="S220" s="3"/>
+      <c r="S220" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T220" s="3"/>
       <c r="U220" s="3"/>
       <c r="V220" s="3"/>
@@ -18156,19 +18158,15 @@
       <c r="Z220" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="AA220" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="AB220" s="3">
-        <v>1</v>
-      </c>
+      <c r="AA220" s="3"/>
+      <c r="AB220" s="3"/>
     </row>
     <row r="221" spans="1:28">
       <c r="A221" s="7">
         <v>219</v>
       </c>
       <c r="B221" s="7">
-        <v>2025102606</v>
+        <v>2025102607</v>
       </c>
       <c r="C221" s="7">
         <v>1</v>
@@ -18207,16 +18205,14 @@
         <v>634</v>
       </c>
       <c r="O221" s="7" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P221" s="7"/>
       <c r="Q221" s="7"/>
       <c r="R221" s="7">
         <v>1291</v>
       </c>
-      <c r="S221" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S221" s="7"/>
       <c r="T221" s="7"/>
       <c r="U221" s="7"/>
       <c r="V221" s="7"/>
@@ -18226,7 +18222,9 @@
       <c r="Z221" s="8" t="s">
         <v>515</v>
       </c>
-      <c r="AA221" s="7"/>
+      <c r="AA221" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="AB221" s="7"/>
     </row>
     <row r="222" spans="1:28">
@@ -18273,7 +18271,7 @@
         <v>602</v>
       </c>
       <c r="O222" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P222" s="3"/>
       <c r="Q222" s="3"/>
@@ -18759,7 +18757,7 @@
         <v>653</v>
       </c>
       <c r="O229" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P229" s="7"/>
       <c r="Q229" s="7">
@@ -18895,7 +18893,7 @@
         <v>657</v>
       </c>
       <c r="O231" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P231" s="7"/>
       <c r="Q231" s="7">
@@ -18967,7 +18965,7 @@
         <v>657</v>
       </c>
       <c r="O232" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P232" s="3"/>
       <c r="Q232" s="3">
@@ -19039,7 +19037,7 @@
         <v>657</v>
       </c>
       <c r="O233" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P233" s="7"/>
       <c r="Q233" s="7">
@@ -19175,7 +19173,7 @@
         <v>634</v>
       </c>
       <c r="O235" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P235" s="7"/>
       <c r="Q235" s="7">
@@ -19311,7 +19309,7 @@
         <v>665</v>
       </c>
       <c r="O237" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P237" s="7"/>
       <c r="Q237" s="7"/>
@@ -19443,7 +19441,7 @@
         <v>668</v>
       </c>
       <c r="O239" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P239" s="7"/>
       <c r="Q239" s="7"/>
@@ -19575,7 +19573,7 @@
         <v>671</v>
       </c>
       <c r="O241" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P241" s="7"/>
       <c r="Q241" s="7"/>
@@ -19707,7 +19705,7 @@
         <v>674</v>
       </c>
       <c r="O243" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P243" s="7"/>
       <c r="Q243" s="7"/>
@@ -19843,7 +19841,7 @@
         <v>677</v>
       </c>
       <c r="O245" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P245" s="7"/>
       <c r="Q245" s="7"/>
@@ -19940,7 +19938,7 @@
         <v>245</v>
       </c>
       <c r="B247" s="7">
-        <v>2025100505</v>
+        <v>2025100506</v>
       </c>
       <c r="C247" s="7">
         <v>1</v>
@@ -19979,16 +19977,14 @@
         <v>668</v>
       </c>
       <c r="O247" s="7" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P247" s="7"/>
       <c r="Q247" s="7"/>
       <c r="R247" s="7">
         <v>187561</v>
       </c>
-      <c r="S247" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S247" s="7"/>
       <c r="T247" s="7"/>
       <c r="U247" s="7"/>
       <c r="V247" s="7"/>
@@ -19998,15 +19994,19 @@
       <c r="Z247" s="8" t="s">
         <v>492</v>
       </c>
-      <c r="AA247" s="7"/>
-      <c r="AB247" s="7"/>
+      <c r="AA247" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB247" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="248" spans="1:28">
       <c r="A248" s="3">
         <v>246</v>
       </c>
       <c r="B248" s="3">
-        <v>2025100506</v>
+        <v>2025100505</v>
       </c>
       <c r="C248" s="3">
         <v>1</v>
@@ -20045,14 +20045,16 @@
         <v>668</v>
       </c>
       <c r="O248" s="3" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P248" s="3"/>
       <c r="Q248" s="3"/>
       <c r="R248" s="3">
         <v>187561</v>
       </c>
-      <c r="S248" s="3"/>
+      <c r="S248" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T248" s="3"/>
       <c r="U248" s="3"/>
       <c r="V248" s="3"/>
@@ -20062,9 +20064,7 @@
       <c r="Z248" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="AA248" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA248" s="3"/>
       <c r="AB248" s="3"/>
     </row>
     <row r="249" spans="1:28">
@@ -20111,7 +20111,7 @@
         <v>682</v>
       </c>
       <c r="O249" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P249" s="7"/>
       <c r="Q249" s="7"/>
@@ -20241,7 +20241,7 @@
       </c>
       <c r="N251" s="8"/>
       <c r="O251" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P251" s="7"/>
       <c r="Q251" s="7"/>
@@ -20373,7 +20373,7 @@
       </c>
       <c r="N253" s="8"/>
       <c r="O253" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P253" s="7"/>
       <c r="Q253" s="7"/>
@@ -20501,7 +20501,7 @@
       </c>
       <c r="N255" s="8"/>
       <c r="O255" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P255" s="7"/>
       <c r="Q255" s="7"/>
@@ -20602,7 +20602,7 @@
         <v>255</v>
       </c>
       <c r="B257" s="7">
-        <v>2025100557</v>
+        <v>2025100558</v>
       </c>
       <c r="C257" s="7">
         <v>1</v>
@@ -20641,7 +20641,7 @@
         <v>532</v>
       </c>
       <c r="O257" s="7" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P257" s="7"/>
       <c r="Q257" s="7">
@@ -20650,9 +20650,7 @@
       <c r="R257" s="7">
         <v>8923</v>
       </c>
-      <c r="S257" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S257" s="7"/>
       <c r="T257" s="7"/>
       <c r="U257" s="7"/>
       <c r="V257" s="7"/>
@@ -20674,7 +20672,7 @@
         <v>256</v>
       </c>
       <c r="B258" s="3">
-        <v>2025100558</v>
+        <v>2025100557</v>
       </c>
       <c r="C258" s="3">
         <v>1</v>
@@ -20713,7 +20711,7 @@
         <v>532</v>
       </c>
       <c r="O258" s="3" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P258" s="3"/>
       <c r="Q258" s="3">
@@ -20722,7 +20720,9 @@
       <c r="R258" s="3">
         <v>8923</v>
       </c>
-      <c r="S258" s="3"/>
+      <c r="S258" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T258" s="3"/>
       <c r="U258" s="3"/>
       <c r="V258" s="3"/>
@@ -20919,7 +20919,7 @@
         <v>590</v>
       </c>
       <c r="O261" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P261" s="7"/>
       <c r="Q261" s="7"/>
@@ -21119,7 +21119,7 @@
         <v>590</v>
       </c>
       <c r="O264" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P264" s="3"/>
       <c r="Q264" s="3"/>
@@ -21325,7 +21325,7 @@
         <v>715</v>
       </c>
       <c r="O267" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P267" s="7"/>
       <c r="Q267" s="7"/>
@@ -21424,7 +21424,7 @@
         <v>267</v>
       </c>
       <c r="B269" s="7">
-        <v>2025100709</v>
+        <v>2025100708</v>
       </c>
       <c r="C269" s="7">
         <v>1</v>
@@ -21463,14 +21463,16 @@
         <v>718</v>
       </c>
       <c r="O269" s="7" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P269" s="7"/>
       <c r="Q269" s="7"/>
       <c r="R269" s="7">
         <v>28</v>
       </c>
-      <c r="S269" s="7"/>
+      <c r="S269" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T269" s="7"/>
       <c r="U269" s="7"/>
       <c r="V269" s="7"/>
@@ -21480,19 +21482,15 @@
       <c r="Z269" s="8" t="s">
         <v>492</v>
       </c>
-      <c r="AA269" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="AB269" s="7">
-        <v>1</v>
-      </c>
+      <c r="AA269" s="7"/>
+      <c r="AB269" s="7"/>
     </row>
     <row r="270" spans="1:28">
       <c r="A270" s="3">
         <v>268</v>
       </c>
       <c r="B270" s="3">
-        <v>2025100708</v>
+        <v>2025100709</v>
       </c>
       <c r="C270" s="3">
         <v>1</v>
@@ -21531,16 +21529,14 @@
         <v>718</v>
       </c>
       <c r="O270" s="3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P270" s="3"/>
       <c r="Q270" s="3"/>
       <c r="R270" s="3">
         <v>28</v>
       </c>
-      <c r="S270" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S270" s="3"/>
       <c r="T270" s="3"/>
       <c r="U270" s="3"/>
       <c r="V270" s="3"/>
@@ -21550,7 +21546,9 @@
       <c r="Z270" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="AA270" s="3"/>
+      <c r="AA270" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="AB270" s="3"/>
     </row>
     <row r="271" spans="1:28">
@@ -21597,7 +21595,7 @@
         <v>671</v>
       </c>
       <c r="O271" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P271" s="7"/>
       <c r="Q271" s="7"/>
@@ -21729,7 +21727,7 @@
         <v>723</v>
       </c>
       <c r="O273" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P273" s="7"/>
       <c r="Q273" s="7"/>
@@ -21867,7 +21865,7 @@
         <v>668</v>
       </c>
       <c r="O275" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P275" s="7"/>
       <c r="Q275" s="7">
@@ -22075,7 +22073,7 @@
         <v>693</v>
       </c>
       <c r="O278" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P278" s="3"/>
       <c r="Q278" s="3"/>
@@ -22147,7 +22145,7 @@
         <v>693</v>
       </c>
       <c r="O279" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P279" s="7"/>
       <c r="Q279" s="7"/>
@@ -22217,7 +22215,7 @@
         <v>693</v>
       </c>
       <c r="O280" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P280" s="3"/>
       <c r="Q280" s="3"/>
@@ -22285,7 +22283,7 @@
         <v>737</v>
       </c>
       <c r="O281" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P281" s="7"/>
       <c r="Q281" s="7"/>
@@ -22355,7 +22353,7 @@
         <v>737</v>
       </c>
       <c r="O282" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P282" s="3"/>
       <c r="Q282" s="3"/>
@@ -22425,7 +22423,7 @@
         <v>737</v>
       </c>
       <c r="O283" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P283" s="7"/>
       <c r="Q283" s="7"/>
@@ -22495,7 +22493,7 @@
         <v>739</v>
       </c>
       <c r="O284" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P284" s="3"/>
       <c r="Q284" s="3"/>
@@ -22565,7 +22563,7 @@
         <v>739</v>
       </c>
       <c r="O285" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P285" s="7"/>
       <c r="Q285" s="7"/>
@@ -22635,7 +22633,7 @@
         <v>739</v>
       </c>
       <c r="O286" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P286" s="3"/>
       <c r="Q286" s="3"/>
@@ -22705,7 +22703,7 @@
         <v>602</v>
       </c>
       <c r="O287" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P287" s="7"/>
       <c r="Q287" s="7"/>
@@ -22802,7 +22800,7 @@
         <v>287</v>
       </c>
       <c r="B289" s="7">
-        <v>2025100079</v>
+        <v>2025100080</v>
       </c>
       <c r="C289" s="7">
         <v>1</v>
@@ -22841,16 +22839,14 @@
         <v>744</v>
       </c>
       <c r="O289" s="7" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="P289" s="7"/>
       <c r="Q289" s="7"/>
       <c r="R289" s="7">
         <v>68795</v>
       </c>
-      <c r="S289" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S289" s="7"/>
       <c r="T289" s="7"/>
       <c r="U289" s="7"/>
       <c r="V289" s="7"/>
@@ -22860,15 +22856,19 @@
       <c r="Z289" s="8" t="s">
         <v>492</v>
       </c>
-      <c r="AA289" s="7"/>
-      <c r="AB289" s="7"/>
+      <c r="AA289" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB289" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="290" spans="1:28">
       <c r="A290" s="3">
         <v>288</v>
       </c>
       <c r="B290" s="3">
-        <v>2025100080</v>
+        <v>2025100079</v>
       </c>
       <c r="C290" s="3">
         <v>1</v>
@@ -22907,14 +22907,16 @@
         <v>744</v>
       </c>
       <c r="O290" s="3" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P290" s="3"/>
       <c r="Q290" s="3"/>
       <c r="R290" s="3">
         <v>68795</v>
       </c>
-      <c r="S290" s="3"/>
+      <c r="S290" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T290" s="3"/>
       <c r="U290" s="3"/>
       <c r="V290" s="3"/>
@@ -22924,9 +22926,7 @@
       <c r="Z290" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="AA290" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA290" s="3"/>
       <c r="AB290" s="3"/>
     </row>
     <row r="291" spans="1:28">
@@ -22973,7 +22973,7 @@
         <v>744</v>
       </c>
       <c r="O291" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P291" s="7"/>
       <c r="Q291" s="7"/>
@@ -23043,7 +23043,7 @@
         <v>746</v>
       </c>
       <c r="O292" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P292" s="3"/>
       <c r="Q292" s="3"/>
@@ -23113,7 +23113,7 @@
         <v>746</v>
       </c>
       <c r="O293" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P293" s="7"/>
       <c r="Q293" s="7"/>
@@ -23183,7 +23183,7 @@
         <v>746</v>
       </c>
       <c r="O294" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P294" s="3"/>
       <c r="Q294" s="3"/>
@@ -23253,7 +23253,7 @@
         <v>751</v>
       </c>
       <c r="O295" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P295" s="7"/>
       <c r="Q295" s="7">
@@ -23389,7 +23389,7 @@
         <v>751</v>
       </c>
       <c r="O297" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P297" s="7"/>
       <c r="Q297" s="7">
@@ -23461,7 +23461,7 @@
         <v>753</v>
       </c>
       <c r="O298" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P298" s="3"/>
       <c r="Q298" s="3">
@@ -23597,7 +23597,7 @@
         <v>753</v>
       </c>
       <c r="O300" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P300" s="3"/>
       <c r="Q300" s="3">
@@ -23665,7 +23665,7 @@
         <v>756</v>
       </c>
       <c r="O301" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P301" s="7"/>
       <c r="Q301" s="7"/>
@@ -23799,7 +23799,7 @@
         <v>759</v>
       </c>
       <c r="O303" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P303" s="7"/>
       <c r="Q303" s="7"/>
@@ -23999,7 +23999,7 @@
         <v>767</v>
       </c>
       <c r="O306" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P306" s="3"/>
       <c r="Q306" s="3"/>
@@ -24063,7 +24063,7 @@
         <v>771</v>
       </c>
       <c r="O307" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P307" s="7"/>
       <c r="Q307" s="7"/>
@@ -24265,7 +24265,7 @@
         <v>779</v>
       </c>
       <c r="O310" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P310" s="3"/>
       <c r="Q310" s="3"/>
@@ -24399,7 +24399,7 @@
         <v>782</v>
       </c>
       <c r="O312" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P312" s="3"/>
       <c r="Q312" s="3"/>
@@ -24665,7 +24665,7 @@
         <v>787</v>
       </c>
       <c r="O316" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P316" s="3"/>
       <c r="Q316" s="3"/>
@@ -24797,7 +24797,7 @@
         <v>792</v>
       </c>
       <c r="O318" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P318" s="3"/>
       <c r="Q318" s="3"/>
@@ -24929,7 +24929,7 @@
         <v>800</v>
       </c>
       <c r="O320" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P320" s="3"/>
       <c r="Q320" s="3"/>
@@ -25063,7 +25063,7 @@
         <v>804</v>
       </c>
       <c r="O322" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P322" s="3"/>
       <c r="Q322" s="3"/>
@@ -25197,7 +25197,7 @@
         <v>808</v>
       </c>
       <c r="O324" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P324" s="3"/>
       <c r="Q324" s="3"/>
@@ -25261,7 +25261,7 @@
         <v>812</v>
       </c>
       <c r="O325" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P325" s="7"/>
       <c r="Q325" s="7"/>
@@ -25329,7 +25329,7 @@
         <v>815</v>
       </c>
       <c r="O326" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P326" s="3"/>
       <c r="Q326" s="3"/>
@@ -25395,7 +25395,7 @@
         <v>815</v>
       </c>
       <c r="O327" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P327" s="7"/>
       <c r="Q327" s="7"/>
@@ -25525,7 +25525,7 @@
         <v>820</v>
       </c>
       <c r="O329" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P329" s="7"/>
       <c r="Q329" s="7"/>
@@ -25593,7 +25593,7 @@
         <v>823</v>
       </c>
       <c r="O330" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P330" s="3"/>
       <c r="Q330" s="3"/>
@@ -25659,7 +25659,7 @@
         <v>827</v>
       </c>
       <c r="O331" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P331" s="7"/>
       <c r="Q331" s="7"/>
@@ -25793,7 +25793,7 @@
         <v>830</v>
       </c>
       <c r="O333" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P333" s="7"/>
       <c r="Q333" s="7"/>
@@ -25927,7 +25927,7 @@
         <v>834</v>
       </c>
       <c r="O335" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P335" s="7"/>
       <c r="Q335" s="7"/>
@@ -26059,7 +26059,7 @@
         <v>840</v>
       </c>
       <c r="O337" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P337" s="7"/>
       <c r="Q337" s="7"/>
@@ -26401,7 +26401,7 @@
         <v>857</v>
       </c>
       <c r="O342" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P342" s="3"/>
       <c r="Q342" s="3"/>
@@ -26533,7 +26533,7 @@
         <v>860</v>
       </c>
       <c r="O344" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P344" s="3"/>
       <c r="Q344" s="3"/>
@@ -26665,7 +26665,7 @@
         <v>863</v>
       </c>
       <c r="O346" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P346" s="3"/>
       <c r="Q346" s="3"/>
@@ -26797,7 +26797,7 @@
         <v>869</v>
       </c>
       <c r="O348" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P348" s="3"/>
       <c r="Q348" s="3"/>
@@ -26867,7 +26867,7 @@
         <v>869</v>
       </c>
       <c r="O349" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P349" s="7"/>
       <c r="Q349" s="7"/>
@@ -27034,7 +27034,7 @@
         <v>350</v>
       </c>
       <c r="B352" s="3">
-        <v>2025102037</v>
+        <v>2025102005</v>
       </c>
       <c r="C352" s="3">
         <v>1</v>
@@ -27057,8 +27057,12 @@
       <c r="I352" s="3" t="s">
         <v>879</v>
       </c>
-      <c r="J352" s="3"/>
-      <c r="K352" s="3"/>
+      <c r="J352" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="K352" s="3" t="s">
+        <v>263</v>
+      </c>
       <c r="L352" s="6" t="s">
         <v>245</v>
       </c>
@@ -27069,16 +27073,14 @@
         <v>881</v>
       </c>
       <c r="O352" s="3" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="P352" s="3"/>
       <c r="Q352" s="3"/>
       <c r="R352" s="3">
         <v>0</v>
       </c>
-      <c r="S352" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S352" s="3"/>
       <c r="T352" s="3"/>
       <c r="U352" s="3"/>
       <c r="V352" s="3"/>
@@ -27086,17 +27088,21 @@
       <c r="X352" s="3"/>
       <c r="Y352" s="3"/>
       <c r="Z352" s="6" t="s">
-        <v>816</v>
-      </c>
-      <c r="AA352" s="3"/>
-      <c r="AB352" s="3"/>
+        <v>882</v>
+      </c>
+      <c r="AA352" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB352" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="353" spans="1:28">
       <c r="A353" s="7">
         <v>351</v>
       </c>
       <c r="B353" s="7">
-        <v>2025102005</v>
+        <v>2025102037</v>
       </c>
       <c r="C353" s="7">
         <v>1</v>
@@ -27119,12 +27125,8 @@
       <c r="I353" s="7" t="s">
         <v>879</v>
       </c>
-      <c r="J353" s="7" t="s">
-        <v>356</v>
-      </c>
-      <c r="K353" s="7" t="s">
-        <v>263</v>
-      </c>
+      <c r="J353" s="7"/>
+      <c r="K353" s="7"/>
       <c r="L353" s="8" t="s">
         <v>245</v>
       </c>
@@ -27135,14 +27137,16 @@
         <v>881</v>
       </c>
       <c r="O353" s="7" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="P353" s="7"/>
       <c r="Q353" s="7"/>
       <c r="R353" s="7">
         <v>0</v>
       </c>
-      <c r="S353" s="7"/>
+      <c r="S353" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T353" s="7"/>
       <c r="U353" s="7"/>
       <c r="V353" s="7"/>
@@ -27150,11 +27154,9 @@
       <c r="X353" s="7"/>
       <c r="Y353" s="7"/>
       <c r="Z353" s="8" t="s">
-        <v>882</v>
-      </c>
-      <c r="AA353" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>816</v>
+      </c>
+      <c r="AA353" s="7"/>
       <c r="AB353" s="7"/>
     </row>
     <row r="354" spans="1:28">
@@ -27197,7 +27199,7 @@
         <v>881</v>
       </c>
       <c r="O354" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P354" s="3"/>
       <c r="Q354" s="3"/>
@@ -27331,7 +27333,7 @@
         <v>894</v>
       </c>
       <c r="O356" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P356" s="3"/>
       <c r="Q356" s="3"/>
@@ -27492,7 +27494,7 @@
         <v>357</v>
       </c>
       <c r="B359" s="7">
-        <v>2025103412</v>
+        <v>2025103385</v>
       </c>
       <c r="C359" s="7">
         <v>1</v>
@@ -27510,10 +27512,10 @@
         <v>250</v>
       </c>
       <c r="H359" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="I359" s="7" t="s">
         <v>900</v>
-      </c>
-      <c r="I359" s="7" t="s">
-        <v>901</v>
       </c>
       <c r="J359" s="7"/>
       <c r="K359" s="7"/>
@@ -27521,13 +27523,13 @@
         <v>245</v>
       </c>
       <c r="M359" s="8" t="s">
+        <v>901</v>
+      </c>
+      <c r="N359" s="8" t="s">
         <v>902</v>
       </c>
-      <c r="N359" s="8" t="s">
-        <v>903</v>
-      </c>
       <c r="O359" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P359" s="7"/>
       <c r="Q359" s="7"/>
@@ -27544,7 +27546,7 @@
       <c r="X359" s="7"/>
       <c r="Y359" s="7"/>
       <c r="Z359" s="8" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="AA359" s="7" t="s">
         <v>40</v>
@@ -27558,7 +27560,7 @@
         <v>358</v>
       </c>
       <c r="B360" s="3">
-        <v>2025103385</v>
+        <v>2025103297</v>
       </c>
       <c r="C360" s="3">
         <v>1</v>
@@ -27576,33 +27578,35 @@
         <v>250</v>
       </c>
       <c r="H360" s="3" t="s">
-        <v>383</v>
+        <v>903</v>
       </c>
       <c r="I360" s="3" t="s">
-        <v>901</v>
-      </c>
-      <c r="J360" s="3"/>
-      <c r="K360" s="3"/>
+        <v>900</v>
+      </c>
+      <c r="J360" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="K360" s="3" t="s">
+        <v>263</v>
+      </c>
       <c r="L360" s="6" t="s">
         <v>245</v>
       </c>
       <c r="M360" s="6" t="s">
+        <v>901</v>
+      </c>
+      <c r="N360" s="6" t="s">
         <v>902</v>
       </c>
-      <c r="N360" s="6" t="s">
-        <v>903</v>
-      </c>
       <c r="O360" s="3" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="P360" s="3"/>
       <c r="Q360" s="3"/>
       <c r="R360" s="3">
         <v>0</v>
       </c>
-      <c r="S360" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S360" s="3"/>
       <c r="T360" s="3"/>
       <c r="U360" s="3"/>
       <c r="V360" s="3"/>
@@ -27610,7 +27614,7 @@
       <c r="X360" s="3"/>
       <c r="Y360" s="3"/>
       <c r="Z360" s="6" t="s">
-        <v>248</v>
+        <v>904</v>
       </c>
       <c r="AA360" s="3" t="s">
         <v>40</v>
@@ -27640,10 +27644,10 @@
         <v>250</v>
       </c>
       <c r="H361" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="I361" s="7" t="s">
         <v>900</v>
-      </c>
-      <c r="I361" s="7" t="s">
-        <v>901</v>
       </c>
       <c r="J361" s="7"/>
       <c r="K361" s="7"/>
@@ -27651,13 +27655,13 @@
         <v>245</v>
       </c>
       <c r="M361" s="8" t="s">
+        <v>901</v>
+      </c>
+      <c r="N361" s="8" t="s">
         <v>902</v>
       </c>
-      <c r="N361" s="8" t="s">
-        <v>903</v>
-      </c>
       <c r="O361" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P361" s="7"/>
       <c r="Q361" s="7"/>
@@ -27674,7 +27678,7 @@
       <c r="X361" s="7"/>
       <c r="Y361" s="7"/>
       <c r="Z361" s="8" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="AA361" s="7" t="s">
         <v>40</v>
@@ -27686,7 +27690,7 @@
         <v>360</v>
       </c>
       <c r="B362" s="3">
-        <v>2025103297</v>
+        <v>2025103412</v>
       </c>
       <c r="C362" s="3">
         <v>1</v>
@@ -27704,35 +27708,33 @@
         <v>250</v>
       </c>
       <c r="H362" s="3" t="s">
+        <v>903</v>
+      </c>
+      <c r="I362" s="3" t="s">
         <v>900</v>
       </c>
-      <c r="I362" s="3" t="s">
-        <v>901</v>
-      </c>
-      <c r="J362" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="K362" s="3" t="s">
-        <v>263</v>
-      </c>
+      <c r="J362" s="3"/>
+      <c r="K362" s="3"/>
       <c r="L362" s="6" t="s">
         <v>245</v>
       </c>
       <c r="M362" s="6" t="s">
+        <v>901</v>
+      </c>
+      <c r="N362" s="6" t="s">
         <v>902</v>
       </c>
-      <c r="N362" s="6" t="s">
-        <v>903</v>
-      </c>
       <c r="O362" s="3" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="P362" s="3"/>
       <c r="Q362" s="3"/>
       <c r="R362" s="3">
         <v>0</v>
       </c>
-      <c r="S362" s="3"/>
+      <c r="S362" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T362" s="3"/>
       <c r="U362" s="3"/>
       <c r="V362" s="3"/>
@@ -27740,7 +27742,7 @@
       <c r="X362" s="3"/>
       <c r="Y362" s="3"/>
       <c r="Z362" s="6" t="s">
-        <v>905</v>
+        <v>255</v>
       </c>
       <c r="AA362" s="3" t="s">
         <v>40</v>
@@ -27914,7 +27916,7 @@
         <v>916</v>
       </c>
       <c r="AB365" s="9">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>